<commit_message>
docs: add portable HTML workshop materials
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/rapp-workshop/downloads/Example Inputs/03 Sample Service Requests.xlsx
+++ b/docs/rapp-workshop/downloads/Example Inputs/03 Sample Service Requests.xlsx
@@ -829,36 +829,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1231,576 +1227,576 @@
   <dimension ref="A1:K16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="2" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="2" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="2" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="K8" s="2" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="J9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="K9" s="2" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="J10" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="K10" s="2" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="J11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="K11" s="2" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="J12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="K12" s="2" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="3" t="s">
+      <c r="J13" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="K13" s="3" t="s">
+      <c r="K13" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="H14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="J14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K14" s="3" t="s">
+      <c r="K14" s="2" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="H15" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J15" s="3" t="s">
+      <c r="J15" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="K15" s="2" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="H16" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="J16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="K16" s="2" t="s">
         <v>116</v>
       </c>
     </row>
@@ -1828,251 +1824,251 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="2" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>156</v>
       </c>
     </row>
@@ -2100,241 +2096,241 @@
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H11"/>
@@ -2366,143 +2362,143 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="2" t="n">
         <f aca="false">COUNTA('Sample Requests'!A2:A200)</f>
         <v>15</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="2" t="n">
         <f aca="false">COUNTIF('Sample Requests'!G2:G200,"Critical")</f>
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="2" t="n">
         <f aca="false">COUNTIF('Sample Requests'!G2:G200,"Unknown")</f>
         <v>2</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B7" s="3" t="n">
-        <f aca="false">COUNTA(unique(filter('Sample Requests'!E2:E200,'Sample Requests'!E2:E200&lt;&gt;"")))</f>
-        <v>1</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="B7" s="2" t="n">
+        <f aca="false">SUMPRODUCT(('Sample Requests'!E2:E200&lt;&gt;"")/COUNTIF('Sample Requests'!E2:E200,'Sample Requests'!E2:E200&amp;""))</f>
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="2" t="n">
         <f aca="false">COUNTIF('Test Prompts'!E2:E200,"Yes")</f>
         <v>8</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="2" t="n">
         <f aca="false">COUNT('Test Prompts'!G2:G200)</f>
         <v>0</v>
       </c>
-      <c r="C9" s="3" t="n">
-        <f aca="false">B7</f>
-        <v>1</v>
-      </c>
-      <c r="D9" s="3" t="s">
+      <c r="C9" s="2" t="n">
+        <f aca="false">COUNTA('Test Prompts'!A2:A200)</f>
+        <v>10</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="6" t="n">
         <f aca="false">IFERROR(AVERAGE('Test Prompts'!G2:G200),0)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>227</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: reframe workshop around local Brainstem
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/rapp-workshop/downloads/Example Inputs/03 Sample Service Requests.xlsx
+++ b/docs/rapp-workshop/downloads/Example Inputs/03 Sample Service Requests.xlsx
@@ -829,32 +829,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1227,576 +1231,576 @@
   <dimension ref="A1:K16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="3" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="3" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="3" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="3" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K7" s="3" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="3" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="3" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="3" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="K11" s="3" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="J12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="K12" s="3" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="J13" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="K13" s="3" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="I14" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="J14" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K14" s="2" t="s">
+      <c r="K14" s="3" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="J15" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="K15" s="3" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="I16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="J16" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="K16" s="3" t="s">
         <v>116</v>
       </c>
     </row>
@@ -1824,251 +1828,251 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="3" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="3" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="3" t="s">
         <v>156</v>
       </c>
     </row>
@@ -2096,241 +2100,241 @@
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H11"/>
@@ -2362,143 +2366,143 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <f aca="false">COUNTA('Sample Requests'!A2:A200)</f>
         <v>15</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <f aca="false">COUNTIF('Sample Requests'!G2:G200,"Critical")</f>
         <v>4</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="3" t="n">
         <f aca="false">COUNTIF('Sample Requests'!G2:G200,"Unknown")</f>
         <v>2</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <f aca="false">SUMPRODUCT(('Sample Requests'!E2:E200&lt;&gt;"")/COUNTIF('Sample Requests'!E2:E200,'Sample Requests'!E2:E200&amp;""))</f>
         <v>8</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <f aca="false">COUNTIF('Test Prompts'!E2:E200,"Yes")</f>
         <v>8</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <f aca="false">COUNT('Test Prompts'!G2:G200)</f>
         <v>0</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="3" t="n">
         <f aca="false">COUNTA('Test Prompts'!A2:A200)</f>
         <v>10</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <f aca="false">IFERROR(AVERAGE('Test Prompts'!G2:G200),0)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>227</v>
       </c>
     </row>

</xml_diff>